<commit_message>
feat(main-console): added filter for fee slab search
</commit_message>
<xml_diff>
--- a/apps/backend/issuereturn_library_migration.xlsx
+++ b/apps/backend/issuereturn_library_migration.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="177">
   <si>
     <t>legacy_id</t>
   </si>
@@ -143,6 +143,405 @@
   </si>
   <si>
     <t>2026-05-14T05:24:04.769Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:07:22.671Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:07:25.131Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:07:26.137Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:07:27.171Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:07:28.167Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:07:29.032Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:07:36.720Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:07:43.053Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:07:44.477Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:07:50.988Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:08:00.606Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:08:09.997Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:08:14.953Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:08:22.718Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:08:27.058Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:08:30.089Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:08:30.797Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:08:36.770Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:08:44.634Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:08:57.647Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:03.377Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:07.479Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:11.331Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:15.512Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:16.296Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:17.064Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:17.820Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:22.891Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:32.476Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:36.853Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:41.281Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:45.247Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:49.152Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:54.329Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:09:57.652Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:10:01.371Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:10:04.887Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:10:08.823Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:10:14.691Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:10:23.512Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:10:29.069Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:10:30.312Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:10:38.201Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:10:43.349Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:10:46.909Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:10:52.967Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:11:01.396Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:11:03.050Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:11:06.221Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:11:12.979Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:11:24.880Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:11:40.445Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:11:48.351Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:12:01.350Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:12:04.839Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:12:08.518Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:12:12.194Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:12:18.813Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:12:30.702Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:12:44.241Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:12:52.101Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:12:53.533Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:13:14.159Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:13:19.216Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:13:51.098Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:13:53.123Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:13:54.710Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:14:00.439Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:14:01.658Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:14:02.831Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:14:07.284Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:14:08.471Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:14:21.617Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:14:28.561Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:15:15.980Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:15:28.039Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:15:50.799Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:15:52.329Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:16:49.457Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:16:59.378Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:17:08.444Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:17:14.862Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:17:20.529Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:17:24.918Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:17:31.210Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:17:36.714Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:17:59.501Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:18:03.484Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:18:04.346Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:18:12.538Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:18:13.621Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:18:23.222Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:18:28.518Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:18:34.830Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:18:35.794Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:18:48.055Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:18:52.188Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:18:55.675Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:18:59.666Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:19:05.027Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:19:18.373Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:19:23.664Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:19:24.492Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:19:25.727Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:19:30.619Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:19:35.760Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:19:36.537Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:19:41.327Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:19:48.414Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:19:53.717Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:19:58.436Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:09.274Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:12.188Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:19.164Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:24.060Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:27.344Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:30.710Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:35.526Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:38.788Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:42.072Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:46.178Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:50.908Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:55.173Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:20:59.166Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:21:02.542Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:21:08.127Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:21:13.188Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:21:19.030Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:21:24.002Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:21:29.033Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:21:32.833Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:21:36.836Z</t>
+  </si>
+  <si>
+    <t>2026-05-16T06:21:44.969Z</t>
   </si>
 </sst>
 </file>
@@ -523,7 +922,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D170"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1044,6 +1443,1868 @@
         <v>43</v>
       </c>
     </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>36130</v>
+      </c>
+      <c r="B38" t="s">
+        <v>13</v>
+      </c>
+      <c r="C38" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>36982</v>
+      </c>
+      <c r="B39" t="s">
+        <v>13</v>
+      </c>
+      <c r="C39" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>37243</v>
+      </c>
+      <c r="B40" t="s">
+        <v>13</v>
+      </c>
+      <c r="C40" t="s">
+        <v>14</v>
+      </c>
+      <c r="D40" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>38017</v>
+      </c>
+      <c r="B41" t="s">
+        <v>13</v>
+      </c>
+      <c r="C41" t="s">
+        <v>14</v>
+      </c>
+      <c r="D41" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>38021</v>
+      </c>
+      <c r="B42" t="s">
+        <v>13</v>
+      </c>
+      <c r="C42" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>39441</v>
+      </c>
+      <c r="B43" t="s">
+        <v>13</v>
+      </c>
+      <c r="C43" t="s">
+        <v>14</v>
+      </c>
+      <c r="D43" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>39797</v>
+      </c>
+      <c r="B44" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" t="s">
+        <v>5</v>
+      </c>
+      <c r="D44" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>39800</v>
+      </c>
+      <c r="B45" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" t="s">
+        <v>5</v>
+      </c>
+      <c r="D45" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>39804</v>
+      </c>
+      <c r="B46" t="s">
+        <v>13</v>
+      </c>
+      <c r="C46" t="s">
+        <v>14</v>
+      </c>
+      <c r="D46" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>39998</v>
+      </c>
+      <c r="B47" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" t="s">
+        <v>5</v>
+      </c>
+      <c r="D47" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>40023</v>
+      </c>
+      <c r="B48" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" t="s">
+        <v>5</v>
+      </c>
+      <c r="D48" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>40024</v>
+      </c>
+      <c r="B49" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" t="s">
+        <v>5</v>
+      </c>
+      <c r="D49" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>40025</v>
+      </c>
+      <c r="B50" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" t="s">
+        <v>5</v>
+      </c>
+      <c r="D50" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>40055</v>
+      </c>
+      <c r="B51" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" t="s">
+        <v>5</v>
+      </c>
+      <c r="D51" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>40701</v>
+      </c>
+      <c r="B52" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" t="s">
+        <v>5</v>
+      </c>
+      <c r="D52" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>40702</v>
+      </c>
+      <c r="B53" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" t="s">
+        <v>5</v>
+      </c>
+      <c r="D53" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>40721</v>
+      </c>
+      <c r="B54" t="s">
+        <v>13</v>
+      </c>
+      <c r="C54" t="s">
+        <v>14</v>
+      </c>
+      <c r="D54" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>40722</v>
+      </c>
+      <c r="B55" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" t="s">
+        <v>5</v>
+      </c>
+      <c r="D55" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>40723</v>
+      </c>
+      <c r="B56" t="s">
+        <v>13</v>
+      </c>
+      <c r="C56" t="s">
+        <v>14</v>
+      </c>
+      <c r="D56" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>40753</v>
+      </c>
+      <c r="B57" t="s">
+        <v>4</v>
+      </c>
+      <c r="C57" t="s">
+        <v>5</v>
+      </c>
+      <c r="D57" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>40754</v>
+      </c>
+      <c r="B58" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" t="s">
+        <v>5</v>
+      </c>
+      <c r="D58" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>40800</v>
+      </c>
+      <c r="B59" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" t="s">
+        <v>5</v>
+      </c>
+      <c r="D59" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>40801</v>
+      </c>
+      <c r="B60" t="s">
+        <v>4</v>
+      </c>
+      <c r="C60" t="s">
+        <v>5</v>
+      </c>
+      <c r="D60" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>40802</v>
+      </c>
+      <c r="B61" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>40996</v>
+      </c>
+      <c r="B62" t="s">
+        <v>13</v>
+      </c>
+      <c r="C62" t="s">
+        <v>14</v>
+      </c>
+      <c r="D62" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>41181</v>
+      </c>
+      <c r="B63" t="s">
+        <v>13</v>
+      </c>
+      <c r="C63" t="s">
+        <v>14</v>
+      </c>
+      <c r="D63" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>41182</v>
+      </c>
+      <c r="B64" t="s">
+        <v>13</v>
+      </c>
+      <c r="C64" t="s">
+        <v>14</v>
+      </c>
+      <c r="D64" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>41301</v>
+      </c>
+      <c r="B65" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" t="s">
+        <v>5</v>
+      </c>
+      <c r="D65" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>41302</v>
+      </c>
+      <c r="B66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C66" t="s">
+        <v>5</v>
+      </c>
+      <c r="D66" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>41406</v>
+      </c>
+      <c r="B67" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" t="s">
+        <v>5</v>
+      </c>
+      <c r="D67" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>41436</v>
+      </c>
+      <c r="B68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" t="s">
+        <v>5</v>
+      </c>
+      <c r="D68" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>41445</v>
+      </c>
+      <c r="B69" t="s">
+        <v>4</v>
+      </c>
+      <c r="C69" t="s">
+        <v>5</v>
+      </c>
+      <c r="D69" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>41456</v>
+      </c>
+      <c r="B70" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" t="s">
+        <v>5</v>
+      </c>
+      <c r="D70" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>41457</v>
+      </c>
+      <c r="B71" t="s">
+        <v>4</v>
+      </c>
+      <c r="C71" t="s">
+        <v>5</v>
+      </c>
+      <c r="D71" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>41458</v>
+      </c>
+      <c r="B72" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" t="s">
+        <v>5</v>
+      </c>
+      <c r="D72" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>41459</v>
+      </c>
+      <c r="B73" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" t="s">
+        <v>5</v>
+      </c>
+      <c r="D73" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>41566</v>
+      </c>
+      <c r="B74" t="s">
+        <v>4</v>
+      </c>
+      <c r="C74" t="s">
+        <v>5</v>
+      </c>
+      <c r="D74" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>41567</v>
+      </c>
+      <c r="B75" t="s">
+        <v>4</v>
+      </c>
+      <c r="C75" t="s">
+        <v>5</v>
+      </c>
+      <c r="D75" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>41568</v>
+      </c>
+      <c r="B76" t="s">
+        <v>4</v>
+      </c>
+      <c r="C76" t="s">
+        <v>5</v>
+      </c>
+      <c r="D76" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>41639</v>
+      </c>
+      <c r="B77" t="s">
+        <v>4</v>
+      </c>
+      <c r="C77" t="s">
+        <v>5</v>
+      </c>
+      <c r="D77" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>41640</v>
+      </c>
+      <c r="B78" t="s">
+        <v>4</v>
+      </c>
+      <c r="C78" t="s">
+        <v>5</v>
+      </c>
+      <c r="D78" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>41696</v>
+      </c>
+      <c r="B79" t="s">
+        <v>13</v>
+      </c>
+      <c r="C79" t="s">
+        <v>14</v>
+      </c>
+      <c r="D79" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>41821</v>
+      </c>
+      <c r="B80" t="s">
+        <v>4</v>
+      </c>
+      <c r="C80" t="s">
+        <v>5</v>
+      </c>
+      <c r="D80" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>41824</v>
+      </c>
+      <c r="B81" t="s">
+        <v>4</v>
+      </c>
+      <c r="C81" t="s">
+        <v>5</v>
+      </c>
+      <c r="D81" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>41850</v>
+      </c>
+      <c r="B82" t="s">
+        <v>4</v>
+      </c>
+      <c r="C82" t="s">
+        <v>5</v>
+      </c>
+      <c r="D82" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>41851</v>
+      </c>
+      <c r="B83" t="s">
+        <v>4</v>
+      </c>
+      <c r="C83" t="s">
+        <v>5</v>
+      </c>
+      <c r="D83" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>41940</v>
+      </c>
+      <c r="B84" t="s">
+        <v>4</v>
+      </c>
+      <c r="C84" t="s">
+        <v>5</v>
+      </c>
+      <c r="D84" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>41952</v>
+      </c>
+      <c r="B85" t="s">
+        <v>13</v>
+      </c>
+      <c r="C85" t="s">
+        <v>14</v>
+      </c>
+      <c r="D85" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>41953</v>
+      </c>
+      <c r="B86" t="s">
+        <v>13</v>
+      </c>
+      <c r="C86" t="s">
+        <v>14</v>
+      </c>
+      <c r="D86" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>41970</v>
+      </c>
+      <c r="B87" t="s">
+        <v>4</v>
+      </c>
+      <c r="C87" t="s">
+        <v>5</v>
+      </c>
+      <c r="D87" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>41971</v>
+      </c>
+      <c r="B88" t="s">
+        <v>4</v>
+      </c>
+      <c r="C88" t="s">
+        <v>5</v>
+      </c>
+      <c r="D88" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>41972</v>
+      </c>
+      <c r="B89" t="s">
+        <v>4</v>
+      </c>
+      <c r="C89" t="s">
+        <v>5</v>
+      </c>
+      <c r="D89" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>41973</v>
+      </c>
+      <c r="B90" t="s">
+        <v>4</v>
+      </c>
+      <c r="C90" t="s">
+        <v>5</v>
+      </c>
+      <c r="D90" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>42066</v>
+      </c>
+      <c r="B91" t="s">
+        <v>4</v>
+      </c>
+      <c r="C91" t="s">
+        <v>5</v>
+      </c>
+      <c r="D91" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>42067</v>
+      </c>
+      <c r="B92" t="s">
+        <v>4</v>
+      </c>
+      <c r="C92" t="s">
+        <v>5</v>
+      </c>
+      <c r="D92" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>42068</v>
+      </c>
+      <c r="B93" t="s">
+        <v>4</v>
+      </c>
+      <c r="C93" t="s">
+        <v>5</v>
+      </c>
+      <c r="D93" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>42102</v>
+      </c>
+      <c r="B94" t="s">
+        <v>4</v>
+      </c>
+      <c r="C94" t="s">
+        <v>5</v>
+      </c>
+      <c r="D94" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>42120</v>
+      </c>
+      <c r="B95" t="s">
+        <v>4</v>
+      </c>
+      <c r="C95" t="s">
+        <v>5</v>
+      </c>
+      <c r="D95" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>42121</v>
+      </c>
+      <c r="B96" t="s">
+        <v>4</v>
+      </c>
+      <c r="C96" t="s">
+        <v>5</v>
+      </c>
+      <c r="D96" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>42258</v>
+      </c>
+      <c r="B97" t="s">
+        <v>4</v>
+      </c>
+      <c r="C97" t="s">
+        <v>5</v>
+      </c>
+      <c r="D97" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>42259</v>
+      </c>
+      <c r="B98" t="s">
+        <v>4</v>
+      </c>
+      <c r="C98" t="s">
+        <v>5</v>
+      </c>
+      <c r="D98" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>42439</v>
+      </c>
+      <c r="B99" t="s">
+        <v>13</v>
+      </c>
+      <c r="C99" t="s">
+        <v>14</v>
+      </c>
+      <c r="D99" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>42526</v>
+      </c>
+      <c r="B100" t="s">
+        <v>4</v>
+      </c>
+      <c r="C100" t="s">
+        <v>5</v>
+      </c>
+      <c r="D100" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>42527</v>
+      </c>
+      <c r="B101" t="s">
+        <v>4</v>
+      </c>
+      <c r="C101" t="s">
+        <v>5</v>
+      </c>
+      <c r="D101" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>42528</v>
+      </c>
+      <c r="B102" t="s">
+        <v>4</v>
+      </c>
+      <c r="C102" t="s">
+        <v>5</v>
+      </c>
+      <c r="D102" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>42669</v>
+      </c>
+      <c r="B103" t="s">
+        <v>13</v>
+      </c>
+      <c r="C103" t="s">
+        <v>14</v>
+      </c>
+      <c r="D103" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>42802</v>
+      </c>
+      <c r="B104" t="s">
+        <v>13</v>
+      </c>
+      <c r="C104" t="s">
+        <v>14</v>
+      </c>
+      <c r="D104" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>42852</v>
+      </c>
+      <c r="B105" t="s">
+        <v>4</v>
+      </c>
+      <c r="C105" t="s">
+        <v>5</v>
+      </c>
+      <c r="D105" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>42854</v>
+      </c>
+      <c r="B106" t="s">
+        <v>13</v>
+      </c>
+      <c r="C106" t="s">
+        <v>14</v>
+      </c>
+      <c r="D106" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>42855</v>
+      </c>
+      <c r="B107" t="s">
+        <v>13</v>
+      </c>
+      <c r="C107" t="s">
+        <v>14</v>
+      </c>
+      <c r="D107" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>42856</v>
+      </c>
+      <c r="B108" t="s">
+        <v>4</v>
+      </c>
+      <c r="C108" t="s">
+        <v>5</v>
+      </c>
+      <c r="D108" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>43251</v>
+      </c>
+      <c r="B109" t="s">
+        <v>13</v>
+      </c>
+      <c r="C109" t="s">
+        <v>14</v>
+      </c>
+      <c r="D109" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>43324</v>
+      </c>
+      <c r="B110" t="s">
+        <v>4</v>
+      </c>
+      <c r="C110" t="s">
+        <v>5</v>
+      </c>
+      <c r="D110" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>43333</v>
+      </c>
+      <c r="B111" t="s">
+        <v>4</v>
+      </c>
+      <c r="C111" t="s">
+        <v>5</v>
+      </c>
+      <c r="D111" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>43439</v>
+      </c>
+      <c r="B112" t="s">
+        <v>4</v>
+      </c>
+      <c r="C112" t="s">
+        <v>5</v>
+      </c>
+      <c r="D112" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>43440</v>
+      </c>
+      <c r="B113" t="s">
+        <v>4</v>
+      </c>
+      <c r="C113" t="s">
+        <v>5</v>
+      </c>
+      <c r="D113" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>43441</v>
+      </c>
+      <c r="B114" t="s">
+        <v>4</v>
+      </c>
+      <c r="C114" t="s">
+        <v>5</v>
+      </c>
+      <c r="D114" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>43620</v>
+      </c>
+      <c r="B115" t="s">
+        <v>13</v>
+      </c>
+      <c r="C115" t="s">
+        <v>14</v>
+      </c>
+      <c r="D115" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>43622</v>
+      </c>
+      <c r="B116" t="s">
+        <v>13</v>
+      </c>
+      <c r="C116" t="s">
+        <v>14</v>
+      </c>
+      <c r="D116" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>43866</v>
+      </c>
+      <c r="B117" t="s">
+        <v>4</v>
+      </c>
+      <c r="C117" t="s">
+        <v>5</v>
+      </c>
+      <c r="D117" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>43867</v>
+      </c>
+      <c r="B118" t="s">
+        <v>4</v>
+      </c>
+      <c r="C118" t="s">
+        <v>5</v>
+      </c>
+      <c r="D118" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>43878</v>
+      </c>
+      <c r="B119" t="s">
+        <v>4</v>
+      </c>
+      <c r="C119" t="s">
+        <v>5</v>
+      </c>
+      <c r="D119" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>43879</v>
+      </c>
+      <c r="B120" t="s">
+        <v>4</v>
+      </c>
+      <c r="C120" t="s">
+        <v>5</v>
+      </c>
+      <c r="D120" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>43934</v>
+      </c>
+      <c r="B121" t="s">
+        <v>4</v>
+      </c>
+      <c r="C121" t="s">
+        <v>5</v>
+      </c>
+      <c r="D121" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>43941</v>
+      </c>
+      <c r="B122" t="s">
+        <v>4</v>
+      </c>
+      <c r="C122" t="s">
+        <v>5</v>
+      </c>
+      <c r="D122" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123">
+        <v>44078</v>
+      </c>
+      <c r="B123" t="s">
+        <v>4</v>
+      </c>
+      <c r="C123" t="s">
+        <v>5</v>
+      </c>
+      <c r="D123" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124">
+        <v>44079</v>
+      </c>
+      <c r="B124" t="s">
+        <v>4</v>
+      </c>
+      <c r="C124" t="s">
+        <v>5</v>
+      </c>
+      <c r="D124" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125">
+        <v>44341</v>
+      </c>
+      <c r="B125" t="s">
+        <v>4</v>
+      </c>
+      <c r="C125" t="s">
+        <v>5</v>
+      </c>
+      <c r="D125" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126">
+        <v>44376</v>
+      </c>
+      <c r="B126" t="s">
+        <v>13</v>
+      </c>
+      <c r="C126" t="s">
+        <v>14</v>
+      </c>
+      <c r="D126" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A127">
+        <v>44456</v>
+      </c>
+      <c r="B127" t="s">
+        <v>4</v>
+      </c>
+      <c r="C127" t="s">
+        <v>5</v>
+      </c>
+      <c r="D127" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128">
+        <v>44632</v>
+      </c>
+      <c r="B128" t="s">
+        <v>13</v>
+      </c>
+      <c r="C128" t="s">
+        <v>14</v>
+      </c>
+      <c r="D128" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A129">
+        <v>44633</v>
+      </c>
+      <c r="B129" t="s">
+        <v>4</v>
+      </c>
+      <c r="C129" t="s">
+        <v>5</v>
+      </c>
+      <c r="D129" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A130">
+        <v>44652</v>
+      </c>
+      <c r="B130" t="s">
+        <v>4</v>
+      </c>
+      <c r="C130" t="s">
+        <v>5</v>
+      </c>
+      <c r="D130" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A131">
+        <v>44653</v>
+      </c>
+      <c r="B131" t="s">
+        <v>4</v>
+      </c>
+      <c r="C131" t="s">
+        <v>5</v>
+      </c>
+      <c r="D131" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A132">
+        <v>44662</v>
+      </c>
+      <c r="B132" t="s">
+        <v>13</v>
+      </c>
+      <c r="C132" t="s">
+        <v>14</v>
+      </c>
+      <c r="D132" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A133">
+        <v>44667</v>
+      </c>
+      <c r="B133" t="s">
+        <v>4</v>
+      </c>
+      <c r="C133" t="s">
+        <v>5</v>
+      </c>
+      <c r="D133" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A134">
+        <v>44668</v>
+      </c>
+      <c r="B134" t="s">
+        <v>4</v>
+      </c>
+      <c r="C134" t="s">
+        <v>5</v>
+      </c>
+      <c r="D134" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A135">
+        <v>44671</v>
+      </c>
+      <c r="B135" t="s">
+        <v>4</v>
+      </c>
+      <c r="C135" t="s">
+        <v>5</v>
+      </c>
+      <c r="D135" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A136">
+        <v>44678</v>
+      </c>
+      <c r="B136" t="s">
+        <v>4</v>
+      </c>
+      <c r="C136" t="s">
+        <v>5</v>
+      </c>
+      <c r="D136" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A137">
+        <v>44679</v>
+      </c>
+      <c r="B137" t="s">
+        <v>4</v>
+      </c>
+      <c r="C137" t="s">
+        <v>5</v>
+      </c>
+      <c r="D137" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A138">
+        <v>44680</v>
+      </c>
+      <c r="B138" t="s">
+        <v>4</v>
+      </c>
+      <c r="C138" t="s">
+        <v>5</v>
+      </c>
+      <c r="D138" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>44699</v>
+      </c>
+      <c r="B139" t="s">
+        <v>4</v>
+      </c>
+      <c r="C139" t="s">
+        <v>5</v>
+      </c>
+      <c r="D139" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>44700</v>
+      </c>
+      <c r="B140" t="s">
+        <v>13</v>
+      </c>
+      <c r="C140" t="s">
+        <v>14</v>
+      </c>
+      <c r="D140" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>44711</v>
+      </c>
+      <c r="B141" t="s">
+        <v>13</v>
+      </c>
+      <c r="C141" t="s">
+        <v>14</v>
+      </c>
+      <c r="D141" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A142">
+        <v>44741</v>
+      </c>
+      <c r="B142" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" t="s">
+        <v>5</v>
+      </c>
+      <c r="D142" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A143">
+        <v>44827</v>
+      </c>
+      <c r="B143" t="s">
+        <v>4</v>
+      </c>
+      <c r="C143" t="s">
+        <v>5</v>
+      </c>
+      <c r="D143" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A144">
+        <v>44859</v>
+      </c>
+      <c r="B144" t="s">
+        <v>13</v>
+      </c>
+      <c r="C144" t="s">
+        <v>14</v>
+      </c>
+      <c r="D144" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A145">
+        <v>44871</v>
+      </c>
+      <c r="B145" t="s">
+        <v>4</v>
+      </c>
+      <c r="C145" t="s">
+        <v>5</v>
+      </c>
+      <c r="D145" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A146">
+        <v>44918</v>
+      </c>
+      <c r="B146" t="s">
+        <v>4</v>
+      </c>
+      <c r="C146" t="s">
+        <v>5</v>
+      </c>
+      <c r="D146" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A147">
+        <v>44919</v>
+      </c>
+      <c r="B147" t="s">
+        <v>4</v>
+      </c>
+      <c r="C147" t="s">
+        <v>5</v>
+      </c>
+      <c r="D147" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A148">
+        <v>45055</v>
+      </c>
+      <c r="B148" t="s">
+        <v>4</v>
+      </c>
+      <c r="C148" t="s">
+        <v>5</v>
+      </c>
+      <c r="D148" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A149">
+        <v>45079</v>
+      </c>
+      <c r="B149" t="s">
+        <v>4</v>
+      </c>
+      <c r="C149" t="s">
+        <v>5</v>
+      </c>
+      <c r="D149" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A150">
+        <v>45080</v>
+      </c>
+      <c r="B150" t="s">
+        <v>4</v>
+      </c>
+      <c r="C150" t="s">
+        <v>5</v>
+      </c>
+      <c r="D150" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A151">
+        <v>45081</v>
+      </c>
+      <c r="B151" t="s">
+        <v>4</v>
+      </c>
+      <c r="C151" t="s">
+        <v>5</v>
+      </c>
+      <c r="D151" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A152">
+        <v>45082</v>
+      </c>
+      <c r="B152" t="s">
+        <v>4</v>
+      </c>
+      <c r="C152" t="s">
+        <v>5</v>
+      </c>
+      <c r="D152" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A153">
+        <v>45097</v>
+      </c>
+      <c r="B153" t="s">
+        <v>4</v>
+      </c>
+      <c r="C153" t="s">
+        <v>5</v>
+      </c>
+      <c r="D153" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A154">
+        <v>45242</v>
+      </c>
+      <c r="B154" t="s">
+        <v>4</v>
+      </c>
+      <c r="C154" t="s">
+        <v>5</v>
+      </c>
+      <c r="D154" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A155">
+        <v>45266</v>
+      </c>
+      <c r="B155" t="s">
+        <v>4</v>
+      </c>
+      <c r="C155" t="s">
+        <v>5</v>
+      </c>
+      <c r="D155" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A156">
+        <v>45276</v>
+      </c>
+      <c r="B156" t="s">
+        <v>4</v>
+      </c>
+      <c r="C156" t="s">
+        <v>5</v>
+      </c>
+      <c r="D156" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A157">
+        <v>45345</v>
+      </c>
+      <c r="B157" t="s">
+        <v>4</v>
+      </c>
+      <c r="C157" t="s">
+        <v>5</v>
+      </c>
+      <c r="D157" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A158">
+        <v>45395</v>
+      </c>
+      <c r="B158" t="s">
+        <v>4</v>
+      </c>
+      <c r="C158" t="s">
+        <v>5</v>
+      </c>
+      <c r="D158" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A159">
+        <v>45396</v>
+      </c>
+      <c r="B159" t="s">
+        <v>4</v>
+      </c>
+      <c r="C159" t="s">
+        <v>5</v>
+      </c>
+      <c r="D159" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A160">
+        <v>45435</v>
+      </c>
+      <c r="B160" t="s">
+        <v>4</v>
+      </c>
+      <c r="C160" t="s">
+        <v>5</v>
+      </c>
+      <c r="D160" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A161">
+        <v>45436</v>
+      </c>
+      <c r="B161" t="s">
+        <v>4</v>
+      </c>
+      <c r="C161" t="s">
+        <v>5</v>
+      </c>
+      <c r="D161" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A162">
+        <v>45444</v>
+      </c>
+      <c r="B162" t="s">
+        <v>4</v>
+      </c>
+      <c r="C162" t="s">
+        <v>5</v>
+      </c>
+      <c r="D162" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A163">
+        <v>45546</v>
+      </c>
+      <c r="B163" t="s">
+        <v>4</v>
+      </c>
+      <c r="C163" t="s">
+        <v>5</v>
+      </c>
+      <c r="D163" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A164">
+        <v>45547</v>
+      </c>
+      <c r="B164" t="s">
+        <v>4</v>
+      </c>
+      <c r="C164" t="s">
+        <v>5</v>
+      </c>
+      <c r="D164" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A165">
+        <v>45600</v>
+      </c>
+      <c r="B165" t="s">
+        <v>4</v>
+      </c>
+      <c r="C165" t="s">
+        <v>5</v>
+      </c>
+      <c r="D165" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A166">
+        <v>45611</v>
+      </c>
+      <c r="B166" t="s">
+        <v>4</v>
+      </c>
+      <c r="C166" t="s">
+        <v>5</v>
+      </c>
+      <c r="D166" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A167">
+        <v>45612</v>
+      </c>
+      <c r="B167" t="s">
+        <v>4</v>
+      </c>
+      <c r="C167" t="s">
+        <v>5</v>
+      </c>
+      <c r="D167" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A168">
+        <v>45655</v>
+      </c>
+      <c r="B168" t="s">
+        <v>4</v>
+      </c>
+      <c r="C168" t="s">
+        <v>5</v>
+      </c>
+      <c r="D168" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A169">
+        <v>45656</v>
+      </c>
+      <c r="B169" t="s">
+        <v>4</v>
+      </c>
+      <c r="C169" t="s">
+        <v>5</v>
+      </c>
+      <c r="D169" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A170">
+        <v>45680</v>
+      </c>
+      <c r="B170" t="s">
+        <v>4</v>
+      </c>
+      <c r="C170" t="s">
+        <v>5</v>
+      </c>
+      <c r="D170" t="s">
+        <v>176</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>